<commit_message>
Update assets and index
</commit_message>
<xml_diff>
--- a/assets/DLR_REIT_Model.xlsx
+++ b/assets/DLR_REIT_Model.xlsx
@@ -44,6 +44,18 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">DLR close 9/30/25 (SEC 8-K). UPDATE to current price before finalizing.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C44" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">APAC held at the same hyperscale cap; Singapore/Tokyo trade tight, offsetting any regional softness.</t>
         </r>
       </text>
     </comment>
@@ -274,7 +286,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="426">
   <si>
     <t xml:space="preserve">Digital Realty (DLR) — Source Data &amp; Reconciliation Anchors</t>
   </si>
@@ -687,7 +699,7 @@
     <t xml:space="preserve">Equity risk premium (ERP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: Damodaran, latest</t>
+    <t xml:space="preserve">Source: Damodaran implied ERP; mid of 4.5-5.5% range</t>
   </si>
   <si>
     <t xml:space="preserve">Beta (vs. XLRE)</t>
@@ -786,13 +798,13 @@
     <t xml:space="preserve">Terminal exit cap rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Current market cap + 50bps</t>
+    <t xml:space="preserve">Stabilized exit cap ~5.75% (CBRE Class-A: 10yr + 100-150bps)</t>
   </si>
   <si>
     <t xml:space="preserve">NAV cap rate — Hyperscale</t>
   </si>
   <si>
-    <t xml:space="preserve">CBRE / Green Street current</t>
+    <t xml:space="preserve">Source: CBRE H2'25 — Class-A ~10yr+100-150bps; ~5.5% for premium hyperscale</t>
   </si>
   <si>
     <t xml:space="preserve">NAV cap rate — Colocation</t>
@@ -1494,7 +1506,7 @@
     <t xml:space="preserve">Recommendation</t>
   </si>
   <si>
-    <t xml:space="preserve">[Buy / Hold / Sell — your call, based on the model output + your thesis]</t>
+    <t xml:space="preserve">HOLD — ~55% premium to stabilized intrinsic (~$131 blended: DCF ~$120, NAV ~$143) with no margin of safety even at the generous corners. The premium reflects development-pipeline and AI-growth optionality a stabilized model excludes; quality asset and structural demand argue for accumulating on power-driven weakness, not chasing at the highs.</t>
   </si>
   <si>
     <t xml:space="preserve">Sensitivity Tables &amp; Output Summary</t>
@@ -1503,25 +1515,19 @@
     <t xml:space="preserve">Two-way sensitivities on the most contested assumptions. Output summary feeds the memo PDF.</t>
   </si>
   <si>
-    <t xml:space="preserve">Two-way tables below: build with Excel Data Table (Data → What-If → Data Table), row input = exit cap / cap rate, column input = WACC / SP-NOI growth, referencing the DCF (B33) &amp; NAV (D57) outputs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SENSITIVITY 1: WACC × Terminal Cap Rate → DCF Value Per Share</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WACC \ Exit Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[link DCF output]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SENSITIVITY 2: SP-NOI Growth × NAV Cap Rate → NAV Per Share</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP-NOI Growth \ Cap Rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[link NAV output]</t>
+    <t xml:space="preserve">Live two-way grids (formula-driven, recalc with the model). S1 = cost of equity x exit cap -&gt; DCF/share. S2 = hyperscale cap x colocation cap -&gt; NAV/share. Base case shaded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SENSITIVITY 1: Cost of Equity x Exit Cap -&gt; DCF Value Per Share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CoE \ Exit cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SENSITIVITY 2: Hyperscale Cap x Colocation Cap -&gt; NAV Per Share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyper cap \ Colo cap</t>
   </si>
   <si>
     <t xml:space="preserve">OUTPUT SUMMARY (for memo)</t>
@@ -1564,7 +1570,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
@@ -1575,8 +1581,10 @@
     <numFmt numFmtId="171" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="172" formatCode="\$#,##0;&quot;($&quot;#,##0&quot;)-&quot;"/>
     <numFmt numFmtId="173" formatCode="0.000"/>
+    <numFmt numFmtId="174" formatCode="0.00%"/>
+    <numFmt numFmtId="175" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1812,14 +1820,6 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <i val="true"/>
-      <sz val="11"/>
-      <color rgb="FFB27D5A"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -1915,7 +1915,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2020,7 +2020,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2072,7 +2072,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2092,7 +2092,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2116,11 +2116,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2128,7 +2128,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2140,7 +2140,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2169,10 +2169,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2208,7 +2204,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2232,12 +2228,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="175" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2714,7 +2718,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="1" t="s">
         <v>53</v>
       </c>
@@ -2743,7 +2747,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="1" t="s">
         <v>60</v>
       </c>
@@ -3133,16 +3137,16 @@
       <c r="A10" s="21" t="s">
         <v>370</v>
       </c>
-      <c r="B10" s="68" t="n">
+      <c r="B10" s="67" t="n">
         <f aca="false">'1. Assumptions'!B31</f>
-        <v>0.1055</v>
+        <v>0.095</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="B11" s="68" t="n">
+      <c r="B11" s="67" t="n">
         <f aca="false">'1. Assumptions'!B32</f>
         <v>0.045</v>
       </c>
@@ -3151,9 +3155,9 @@
       <c r="A12" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="B12" s="69" t="n">
+      <c r="B12" s="68" t="n">
         <f aca="false">'1. Assumptions'!B34</f>
-        <v>0.078275</v>
+        <v>0.0725</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3185,27 +3189,27 @@
       <c r="A17" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="B17" s="70" t="n">
+      <c r="B17" s="69" t="n">
         <f aca="false">'8. FFO-AFFO'!$N$5*(1+'1. Assumptions'!$G$28)</f>
         <v>7.94425</v>
       </c>
-      <c r="C17" s="70" t="n">
+      <c r="C17" s="69" t="n">
         <f aca="false">B17*(1+'1. Assumptions'!$H$28)</f>
         <v>8.420905</v>
       </c>
-      <c r="D17" s="70" t="n">
+      <c r="D17" s="69" t="n">
         <f aca="false">C17*(1+'1. Assumptions'!$I$28)</f>
         <v>8.84195025</v>
       </c>
-      <c r="E17" s="70" t="n">
+      <c r="E17" s="69" t="n">
         <f aca="false">D17*(1+'1. Assumptions'!$J$28)</f>
         <v>9.2840477625</v>
       </c>
-      <c r="F17" s="70" t="n">
+      <c r="F17" s="69" t="n">
         <f aca="false">E17*(1+'1. Assumptions'!$K$28)</f>
         <v>9.655409673</v>
       </c>
-      <c r="G17" s="70" t="n">
+      <c r="G17" s="69" t="n">
         <f aca="false">F17*(1+'1. Assumptions'!$B$12)</f>
         <v>9.896794914825</v>
       </c>
@@ -3214,27 +3218,27 @@
       <c r="A18" s="21" t="s">
         <v>354</v>
       </c>
-      <c r="B18" s="71" t="n">
+      <c r="B18" s="70" t="n">
         <f aca="false">B17*'8. FFO-AFFO'!$N$8*'1. Assumptions'!$B$38</f>
         <v>2418.86524</v>
       </c>
-      <c r="C18" s="71" t="n">
+      <c r="C18" s="70" t="n">
         <f aca="false">C17*'8. FFO-AFFO'!$N$8*'1. Assumptions'!$B$38</f>
         <v>2563.9971544</v>
       </c>
-      <c r="D18" s="71" t="n">
+      <c r="D18" s="70" t="n">
         <f aca="false">D17*'8. FFO-AFFO'!$N$8*'1. Assumptions'!$B$38</f>
         <v>2692.19701212</v>
       </c>
-      <c r="E18" s="71" t="n">
+      <c r="E18" s="70" t="n">
         <f aca="false">E17*'8. FFO-AFFO'!$N$8*'1. Assumptions'!$B$38</f>
         <v>2826.806862726</v>
       </c>
-      <c r="F18" s="71" t="n">
+      <c r="F18" s="70" t="n">
         <f aca="false">F17*'8. FFO-AFFO'!$N$8*'1. Assumptions'!$B$38</f>
         <v>2939.87913723504</v>
       </c>
-      <c r="G18" s="71" t="n">
+      <c r="G18" s="70" t="n">
         <f aca="false">G17*'8. FFO-AFFO'!$N$8*'1. Assumptions'!$B$38</f>
         <v>3013.37611566592</v>
       </c>
@@ -3243,23 +3247,23 @@
       <c r="A19" s="21" t="s">
         <v>373</v>
       </c>
-      <c r="B19" s="71" t="n">
+      <c r="B19" s="70" t="n">
         <f aca="false">-'1. Assumptions'!G23</f>
         <v>-800</v>
       </c>
-      <c r="C19" s="71" t="n">
+      <c r="C19" s="70" t="n">
         <f aca="false">-'1. Assumptions'!H23</f>
         <v>-1000</v>
       </c>
-      <c r="D19" s="71" t="n">
+      <c r="D19" s="70" t="n">
         <f aca="false">-'1. Assumptions'!I23</f>
         <v>-1200</v>
       </c>
-      <c r="E19" s="71" t="n">
+      <c r="E19" s="70" t="n">
         <f aca="false">-'1. Assumptions'!J23</f>
         <v>-1300</v>
       </c>
-      <c r="F19" s="71" t="n">
+      <c r="F19" s="70" t="n">
         <f aca="false">-'1. Assumptions'!K23</f>
         <v>-1100</v>
       </c>
@@ -3269,23 +3273,23 @@
       <c r="A20" s="21" t="s">
         <v>374</v>
       </c>
-      <c r="B20" s="71" t="n">
+      <c r="B20" s="70" t="n">
         <f aca="false">-B19*'1. Assumptions'!$B$39</f>
         <v>400</v>
       </c>
-      <c r="C20" s="71" t="n">
+      <c r="C20" s="70" t="n">
         <f aca="false">-C19*'1. Assumptions'!$B$39</f>
         <v>500</v>
       </c>
-      <c r="D20" s="71" t="n">
+      <c r="D20" s="70" t="n">
         <f aca="false">-D19*'1. Assumptions'!$B$39</f>
         <v>600</v>
       </c>
-      <c r="E20" s="71" t="n">
+      <c r="E20" s="70" t="n">
         <f aca="false">-E19*'1. Assumptions'!$B$39</f>
         <v>650</v>
       </c>
-      <c r="F20" s="71" t="n">
+      <c r="F20" s="70" t="n">
         <f aca="false">-F19*'1. Assumptions'!$B$39</f>
         <v>550</v>
       </c>
@@ -3295,23 +3299,23 @@
       <c r="A21" s="32" t="s">
         <v>375</v>
       </c>
-      <c r="B21" s="71" t="n">
+      <c r="B21" s="70" t="n">
         <f aca="false">B18+B19+B20</f>
         <v>2018.86524</v>
       </c>
-      <c r="C21" s="71" t="n">
+      <c r="C21" s="70" t="n">
         <f aca="false">C18+C19+C20</f>
         <v>2063.9971544</v>
       </c>
-      <c r="D21" s="71" t="n">
+      <c r="D21" s="70" t="n">
         <f aca="false">D18+D19+D20</f>
         <v>2092.19701212</v>
       </c>
-      <c r="E21" s="71" t="n">
+      <c r="E21" s="70" t="n">
         <f aca="false">E18+E19+E20</f>
         <v>2176.806862726</v>
       </c>
-      <c r="F21" s="71" t="n">
+      <c r="F21" s="70" t="n">
         <f aca="false">F18+F19+F20</f>
         <v>2389.87913723504</v>
       </c>
@@ -3321,51 +3325,51 @@
       <c r="A22" s="21" t="s">
         <v>376</v>
       </c>
-      <c r="B22" s="72" t="n">
+      <c r="B22" s="71" t="n">
         <f aca="false">1/(1+'1. Assumptions'!$B$31)^1</f>
-        <v>0.904568068747173</v>
-      </c>
-      <c r="C22" s="72" t="n">
+        <v>0.91324200913242</v>
+      </c>
+      <c r="C22" s="71" t="n">
         <f aca="false">1/(1+'1. Assumptions'!$B$31)^2</f>
-        <v>0.818243390996991</v>
-      </c>
-      <c r="D22" s="72" t="n">
+        <v>0.834010967244219</v>
+      </c>
+      <c r="D22" s="71" t="n">
         <f aca="false">1/(1+'1. Assumptions'!$B$31)^3</f>
-        <v>0.740156843959286</v>
-      </c>
-      <c r="E22" s="72" t="n">
+        <v>0.761653851364584</v>
+      </c>
+      <c r="E22" s="71" t="n">
         <f aca="false">1/(1+'1. Assumptions'!$B$31)^4</f>
-        <v>0.669522246910254</v>
-      </c>
-      <c r="F22" s="72" t="n">
+        <v>0.695574293483638</v>
+      </c>
+      <c r="F22" s="71" t="n">
         <f aca="false">1/(1+'1. Assumptions'!$B$31)^5</f>
-        <v>0.605628445870877</v>
-      </c>
-      <c r="G22" s="72"/>
+        <v>0.635227665281862</v>
+      </c>
+      <c r="G22" s="71"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
         <v>377</v>
       </c>
-      <c r="B23" s="71" t="n">
+      <c r="B23" s="70" t="n">
         <f aca="false">B21*B22</f>
-        <v>1826.2010312076</v>
-      </c>
-      <c r="C23" s="71" t="n">
+        <v>1843.71254794521</v>
+      </c>
+      <c r="C23" s="70" t="n">
         <f aca="false">C21*C22</f>
-        <v>1688.8520306244</v>
-      </c>
-      <c r="D23" s="71" t="n">
+        <v>1721.39626313046</v>
+      </c>
+      <c r="D23" s="70" t="n">
         <f aca="false">D21*D22</f>
-        <v>1548.55393743179</v>
-      </c>
-      <c r="E23" s="71" t="n">
+        <v>1593.52991209467</v>
+      </c>
+      <c r="E23" s="70" t="n">
         <f aca="false">E21*E22</f>
-        <v>1457.42062182197</v>
-      </c>
-      <c r="F23" s="71" t="n">
+        <v>1514.13089559097</v>
+      </c>
+      <c r="F23" s="70" t="n">
         <f aca="false">F21*F22</f>
-        <v>1447.37878770289</v>
+        <v>1518.11734465164</v>
       </c>
       <c r="G23" s="40"/>
     </row>
@@ -3373,9 +3377,9 @@
       <c r="A26" s="21" t="s">
         <v>378</v>
       </c>
-      <c r="G26" s="71" t="n">
+      <c r="G26" s="70" t="n">
         <f aca="false">G18/'1. Assumptions'!$B$35</f>
-        <v>46359.6325487064</v>
+        <v>52406.5411420159</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3384,7 +3388,7 @@
       </c>
       <c r="G27" s="56" t="n">
         <f aca="false">G26*F22</f>
-        <v>28076.712211618</v>
+        <v>33290.0847751406</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3393,7 +3397,7 @@
       </c>
       <c r="B28" s="56" t="n">
         <f aca="false">SUM(B23:F23)</f>
-        <v>7968.40640878864</v>
+        <v>8190.88696341296</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3402,7 +3406,7 @@
       </c>
       <c r="B29" s="56" t="n">
         <f aca="false">G27</f>
-        <v>28076.712211618</v>
+        <v>33290.0847751406</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3411,14 +3415,14 @@
       </c>
       <c r="B30" s="56" t="n">
         <f aca="false">B28+B29</f>
-        <v>36045.1186204066</v>
+        <v>41480.9717385536</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
         <v>325</v>
       </c>
-      <c r="B31" s="73" t="n">
+      <c r="B31" s="72" t="n">
         <f aca="false">'8. FFO-AFFO'!$N$8</f>
         <v>346</v>
       </c>
@@ -3427,15 +3431,15 @@
       <c r="A32" s="21"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="74" t="s">
+      <c r="A33" s="73" t="s">
         <v>383</v>
       </c>
-      <c r="B33" s="75" t="n">
+      <c r="B33" s="74" t="n">
         <f aca="false">IFERROR(B30/B31,0)</f>
-        <v>104.17664341158</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>119.887201556513</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="44" t="s">
         <v>384</v>
       </c>
@@ -3481,12 +3485,13 @@
         <f aca="false">'3. Segment Build'!G17</f>
         <v>1792.2</v>
       </c>
-      <c r="C42" s="22" t="n">
-        <v>0.065</v>
+      <c r="C42" s="67" t="n">
+        <f aca="false">'1. Assumptions'!B36</f>
+        <v>0.055</v>
       </c>
       <c r="D42" s="40" t="n">
         <f aca="false">B42/C42</f>
-        <v>27572.3076923077</v>
+        <v>32585.4545454545</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3497,12 +3502,13 @@
         <f aca="false">'3. Segment Build'!G18</f>
         <v>1014.75</v>
       </c>
-      <c r="C43" s="22" t="n">
-        <v>0.065</v>
+      <c r="C43" s="67" t="n">
+        <f aca="false">'1. Assumptions'!B36</f>
+        <v>0.055</v>
       </c>
       <c r="D43" s="40" t="n">
         <f aca="false">B43/C43</f>
-        <v>15611.5384615385</v>
+        <v>18450</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3513,12 +3519,13 @@
         <f aca="false">'3. Segment Build'!G19</f>
         <v>592.8</v>
       </c>
-      <c r="C44" s="22" t="n">
-        <v>0.07</v>
+      <c r="C44" s="67" t="n">
+        <f aca="false">'1. Assumptions'!B36</f>
+        <v>0.055</v>
       </c>
       <c r="D44" s="40" t="n">
         <f aca="false">B44/C44</f>
-        <v>8468.57142857143</v>
+        <v>10778.1818181818</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3529,7 +3536,8 @@
         <f aca="false">'3. Segment Build'!G20</f>
         <v>373.32</v>
       </c>
-      <c r="C45" s="22" t="n">
+      <c r="C45" s="67" t="n">
+        <f aca="false">'1. Assumptions'!B37</f>
         <v>0.06</v>
       </c>
       <c r="D45" s="40" t="n">
@@ -3541,12 +3549,12 @@
       <c r="A47" s="32" t="s">
         <v>391</v>
       </c>
-      <c r="D47" s="76" t="n">
+      <c r="D47" s="75" t="n">
         <f aca="false">SUM(D42:D45)</f>
-        <v>57874.4175824176</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>68035.6363636364</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="44" t="s">
         <v>392</v>
       </c>
@@ -3592,7 +3600,7 @@
       </c>
       <c r="D54" s="41" t="n">
         <f aca="false">D47+D49+D50-D51-D52</f>
-        <v>39174.4175824176</v>
+        <v>49335.6363636364</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3608,9 +3616,9 @@
       <c r="A57" s="32" t="s">
         <v>398</v>
       </c>
-      <c r="D57" s="77" t="n">
+      <c r="D57" s="76" t="n">
         <f aca="false">IFERROR(D54/D55,0)</f>
-        <v>113.220860064791</v>
+        <v>142.588544403573</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3633,7 +3641,7 @@
       </c>
       <c r="B64" s="62" t="n">
         <f aca="false">B33</f>
-        <v>104.17664341158</v>
+        <v>119.887201556513</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3642,40 +3650,40 @@
       </c>
       <c r="B65" s="62" t="n">
         <f aca="false">D57</f>
-        <v>113.220860064791</v>
+        <v>142.588544403573</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="21" t="s">
         <v>402</v>
       </c>
-      <c r="B66" s="64" t="n">
-        <v>172.88</v>
+      <c r="B66" s="51" t="n">
+        <v>203.62</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="32" t="s">
         <v>403</v>
       </c>
-      <c r="B68" s="77" t="n">
+      <c r="B68" s="76" t="n">
         <f aca="false">AVERAGE(B64:B65)</f>
-        <v>108.698751738185</v>
+        <v>131.237872980043</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="32" t="s">
         <v>404</v>
       </c>
-      <c r="B70" s="78" t="n">
+      <c r="B70" s="77" t="n">
         <f aca="false">IFERROR(B68/B66-1,0)</f>
-        <v>-0.37124738698412</v>
+        <v>-0.355476510264005</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="32" t="s">
         <v>405</v>
       </c>
-      <c r="B72" s="79" t="s">
+      <c r="B72" s="57" t="s">
         <v>406</v>
       </c>
     </row>
@@ -3714,7 +3722,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="44" t="s">
         <v>409</v>
       </c>
@@ -3735,125 +3743,150 @@
       <c r="A9" s="32" t="s">
         <v>411</v>
       </c>
-      <c r="B9" s="80" t="n">
+      <c r="B9" s="78" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C9" s="78" t="n">
         <v>0.055</v>
       </c>
-      <c r="C9" s="80" t="n">
+      <c r="D9" s="78" t="n">
+        <v>0.0575</v>
+      </c>
+      <c r="E9" s="78" t="n">
         <v>0.06</v>
       </c>
-      <c r="D9" s="80" t="n">
+      <c r="F9" s="78" t="n">
         <v>0.065</v>
       </c>
-      <c r="E9" s="80" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="F9" s="80" t="n">
-        <v>0.075</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="78" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="B10" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="C10" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="D10" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="E10" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="F10" s="62" t="s">
-        <v>412</v>
+      <c r="A10" s="79" t="n">
+        <v>0.085</v>
+      </c>
+      <c r="B10" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A10)^1+'9. Valuation'!$C$21/(1+$A10)^2+'9. Valuation'!$D$21/(1+$A10)^3+'9. Valuation'!$E$21/(1+$A10)^4+'9. Valuation'!$F$21/(1+$A10)^5+('9. Valuation'!$G$18/B$9)/(1+$A10)^5)/'9. Valuation'!$B$31</f>
+        <v>140.152377147866</v>
+      </c>
+      <c r="C10" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A10)^1+'9. Valuation'!$C$21/(1+$A10)^2+'9. Valuation'!$D$21/(1+$A10)^3+'9. Valuation'!$E$21/(1+$A10)^4+'9. Valuation'!$F$21/(1+$A10)^5+('9. Valuation'!$G$18/C$9)/(1+$A10)^5)/'9. Valuation'!$B$31</f>
+        <v>129.62146808654</v>
+      </c>
+      <c r="D10" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A10)^1+'9. Valuation'!$C$21/(1+$A10)^2+'9. Valuation'!$D$21/(1+$A10)^3+'9. Valuation'!$E$21/(1+$A10)^4+'9. Valuation'!$F$21/(1+$A10)^5+('9. Valuation'!$G$18/D$9)/(1+$A10)^5)/'9. Valuation'!$B$31</f>
+        <v>125.04281197292</v>
+      </c>
+      <c r="E10" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A10)^1+'9. Valuation'!$C$21/(1+$A10)^2+'9. Valuation'!$D$21/(1+$A10)^3+'9. Valuation'!$E$21/(1+$A10)^4+'9. Valuation'!$F$21/(1+$A10)^5+('9. Valuation'!$G$18/E$9)/(1+$A10)^5)/'9. Valuation'!$B$31</f>
+        <v>120.845710535435</v>
+      </c>
+      <c r="F10" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A10)^1+'9. Valuation'!$C$21/(1+$A10)^2+'9. Valuation'!$D$21/(1+$A10)^3+'9. Valuation'!$E$21/(1+$A10)^4+'9. Valuation'!$F$21/(1+$A10)^5+('9. Valuation'!$G$18/F$9)/(1+$A10)^5)/'9. Valuation'!$B$31</f>
+        <v>113.420069530654</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="78" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="B11" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="C11" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="D11" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="E11" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="F11" s="62" t="s">
-        <v>412</v>
+      <c r="A11" s="79" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="B11" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A11)^1+'9. Valuation'!$C$21/(1+$A11)^2+'9. Valuation'!$D$21/(1+$A11)^3+'9. Valuation'!$E$21/(1+$A11)^4+'9. Valuation'!$F$21/(1+$A11)^5+('9. Valuation'!$G$18/B$9)/(1+$A11)^5)/'9. Valuation'!$B$31</f>
+        <v>137.196738940893</v>
+      </c>
+      <c r="C11" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A11)^1+'9. Valuation'!$C$21/(1+$A11)^2+'9. Valuation'!$D$21/(1+$A11)^3+'9. Valuation'!$E$21/(1+$A11)^4+'9. Valuation'!$F$21/(1+$A11)^5+('9. Valuation'!$G$18/C$9)/(1+$A11)^5)/'9. Valuation'!$B$31</f>
+        <v>126.905158718648</v>
+      </c>
+      <c r="D11" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A11)^1+'9. Valuation'!$C$21/(1+$A11)^2+'9. Valuation'!$D$21/(1+$A11)^3+'9. Valuation'!$E$21/(1+$A11)^4+'9. Valuation'!$F$21/(1+$A11)^5+('9. Valuation'!$G$18/D$9)/(1+$A11)^5)/'9. Valuation'!$B$31</f>
+        <v>122.43055862202</v>
+      </c>
+      <c r="E11" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A11)^1+'9. Valuation'!$C$21/(1+$A11)^2+'9. Valuation'!$D$21/(1+$A11)^3+'9. Valuation'!$E$21/(1+$A11)^4+'9. Valuation'!$F$21/(1+$A11)^5+('9. Valuation'!$G$18/E$9)/(1+$A11)^5)/'9. Valuation'!$B$31</f>
+        <v>118.328841866778</v>
+      </c>
+      <c r="F11" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A11)^1+'9. Valuation'!$C$21/(1+$A11)^2+'9. Valuation'!$D$21/(1+$A11)^3+'9. Valuation'!$E$21/(1+$A11)^4+'9. Valuation'!$F$21/(1+$A11)^5+('9. Valuation'!$G$18/F$9)/(1+$A11)^5)/'9. Valuation'!$B$31</f>
+        <v>111.071958376734</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="78" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="B12" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="C12" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="D12" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="E12" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="F12" s="62" t="s">
-        <v>412</v>
+      <c r="A12" s="79" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="B12" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A12)^1+'9. Valuation'!$C$21/(1+$A12)^2+'9. Valuation'!$D$21/(1+$A12)^3+'9. Valuation'!$E$21/(1+$A12)^4+'9. Valuation'!$F$21/(1+$A12)^5+('9. Valuation'!$G$18/B$9)/(1+$A12)^5)/'9. Valuation'!$B$31</f>
+        <v>134.319319233597</v>
+      </c>
+      <c r="C12" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A12)^1+'9. Valuation'!$C$21/(1+$A12)^2+'9. Valuation'!$D$21/(1+$A12)^3+'9. Valuation'!$E$21/(1+$A12)^4+'9. Valuation'!$F$21/(1+$A12)^5+('9. Valuation'!$G$18/C$9)/(1+$A12)^5)/'9. Valuation'!$B$31</f>
+        <v>124.260570549569</v>
+      </c>
+      <c r="D12" s="81" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A12)^1+'9. Valuation'!$C$21/(1+$A12)^2+'9. Valuation'!$D$21/(1+$A12)^3+'9. Valuation'!$E$21/(1+$A12)^4+'9. Valuation'!$F$21/(1+$A12)^5+('9. Valuation'!$G$18/D$9)/(1+$A12)^5)/'9. Valuation'!$B$31</f>
+        <v>119.887201556513</v>
+      </c>
+      <c r="E12" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A12)^1+'9. Valuation'!$C$21/(1+$A12)^2+'9. Valuation'!$D$21/(1+$A12)^3+'9. Valuation'!$E$21/(1+$A12)^4+'9. Valuation'!$F$21/(1+$A12)^5+('9. Valuation'!$G$18/E$9)/(1+$A12)^5)/'9. Valuation'!$B$31</f>
+        <v>115.878279979545</v>
+      </c>
+      <c r="F12" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A12)^1+'9. Valuation'!$C$21/(1+$A12)^2+'9. Valuation'!$D$21/(1+$A12)^3+'9. Valuation'!$E$21/(1+$A12)^4+'9. Valuation'!$F$21/(1+$A12)^5+('9. Valuation'!$G$18/F$9)/(1+$A12)^5)/'9. Valuation'!$B$31</f>
+        <v>108.785572574141</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="78" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="B13" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="C13" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="D13" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="E13" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="F13" s="62" t="s">
-        <v>412</v>
+      <c r="A13" s="79" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B13" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A13)^1+'9. Valuation'!$C$21/(1+$A13)^2+'9. Valuation'!$D$21/(1+$A13)^3+'9. Valuation'!$E$21/(1+$A13)^4+'9. Valuation'!$F$21/(1+$A13)^5+('9. Valuation'!$G$18/B$9)/(1+$A13)^5)/'9. Valuation'!$B$31</f>
+        <v>131.517683165613</v>
+      </c>
+      <c r="C13" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A13)^1+'9. Valuation'!$C$21/(1+$A13)^2+'9. Valuation'!$D$21/(1+$A13)^3+'9. Valuation'!$E$21/(1+$A13)^4+'9. Valuation'!$F$21/(1+$A13)^5+('9. Valuation'!$G$18/C$9)/(1+$A13)^5)/'9. Valuation'!$B$31</f>
+        <v>121.685473577519</v>
+      </c>
+      <c r="D13" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A13)^1+'9. Valuation'!$C$21/(1+$A13)^2+'9. Valuation'!$D$21/(1+$A13)^3+'9. Valuation'!$E$21/(1+$A13)^4+'9. Valuation'!$F$21/(1+$A13)^5+('9. Valuation'!$G$18/D$9)/(1+$A13)^5)/'9. Valuation'!$B$31</f>
+        <v>117.410599843566</v>
+      </c>
+      <c r="E13" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A13)^1+'9. Valuation'!$C$21/(1+$A13)^2+'9. Valuation'!$D$21/(1+$A13)^3+'9. Valuation'!$E$21/(1+$A13)^4+'9. Valuation'!$F$21/(1+$A13)^5+('9. Valuation'!$G$18/E$9)/(1+$A13)^5)/'9. Valuation'!$B$31</f>
+        <v>113.491965587442</v>
+      </c>
+      <c r="F13" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A13)^1+'9. Valuation'!$C$21/(1+$A13)^2+'9. Valuation'!$D$21/(1+$A13)^3+'9. Valuation'!$E$21/(1+$A13)^4+'9. Valuation'!$F$21/(1+$A13)^5+('9. Valuation'!$G$18/F$9)/(1+$A13)^5)/'9. Valuation'!$B$31</f>
+        <v>106.558997288145</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="78" t="n">
-        <v>0.085</v>
-      </c>
-      <c r="B14" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="C14" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="D14" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="E14" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="F14" s="62" t="s">
-        <v>412</v>
+      <c r="A14" s="79" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="B14" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A14)^1+'9. Valuation'!$C$21/(1+$A14)^2+'9. Valuation'!$D$21/(1+$A14)^3+'9. Valuation'!$E$21/(1+$A14)^4+'9. Valuation'!$F$21/(1+$A14)^5+('9. Valuation'!$G$18/B$9)/(1+$A14)^5)/'9. Valuation'!$B$31</f>
+        <v>128.789482552743</v>
+      </c>
+      <c r="C14" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A14)^1+'9. Valuation'!$C$21/(1+$A14)^2+'9. Valuation'!$D$21/(1+$A14)^3+'9. Valuation'!$E$21/(1+$A14)^4+'9. Valuation'!$F$21/(1+$A14)^5+('9. Valuation'!$G$18/C$9)/(1+$A14)^5)/'9. Valuation'!$B$31</f>
+        <v>119.177717128154</v>
+      </c>
+      <c r="D14" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A14)^1+'9. Valuation'!$C$21/(1+$A14)^2+'9. Valuation'!$D$21/(1+$A14)^3+'9. Valuation'!$E$21/(1+$A14)^4+'9. Valuation'!$F$21/(1+$A14)^5+('9. Valuation'!$G$18/D$9)/(1+$A14)^5)/'9. Valuation'!$B$31</f>
+        <v>114.99868868268</v>
+      </c>
+      <c r="E14" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A14)^1+'9. Valuation'!$C$21/(1+$A14)^2+'9. Valuation'!$D$21/(1+$A14)^3+'9. Valuation'!$E$21/(1+$A14)^4+'9. Valuation'!$F$21/(1+$A14)^5+('9. Valuation'!$G$18/E$9)/(1+$A14)^5)/'9. Valuation'!$B$31</f>
+        <v>111.167912607663</v>
+      </c>
+      <c r="F14" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$21/(1+$A14)^1+'9. Valuation'!$C$21/(1+$A14)^2+'9. Valuation'!$D$21/(1+$A14)^3+'9. Valuation'!$E$21/(1+$A14)^4+'9. Valuation'!$F$21/(1+$A14)^5+('9. Valuation'!$G$18/F$9)/(1+$A14)^5)/'9. Valuation'!$B$31</f>
+        <v>104.390385705708</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
@@ -3865,127 +3898,118 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>414</v>
-      </c>
-      <c r="B21" s="78" t="n">
+        <v>413</v>
+      </c>
+      <c r="B21" s="79" t="n">
         <v>0.055</v>
       </c>
-      <c r="C21" s="78" t="n">
+      <c r="C21" s="79" t="n">
         <v>0.06</v>
       </c>
-      <c r="D21" s="78" t="n">
+      <c r="D21" s="79" t="n">
         <v>0.065</v>
       </c>
-      <c r="E21" s="78" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="F21" s="78" t="n">
-        <v>0.075</v>
-      </c>
+      <c r="E21" s="77"/>
+      <c r="F21" s="77"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="78" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="E22" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="F22" s="21" t="s">
-        <v>415</v>
-      </c>
+      <c r="A22" s="79" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="B22" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A22+'9. Valuation'!$B$43/$A22+'9. Valuation'!$B$44/$A22+'9. Valuation'!$B$45/B$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>162.088544403573</v>
+      </c>
+      <c r="C22" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A22+'9. Valuation'!$B$43/$A22+'9. Valuation'!$B$44/$A22+'9. Valuation'!$B$45/C$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>160.453757225434</v>
+      </c>
+      <c r="D22" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A22+'9. Valuation'!$B$43/$A22+'9. Valuation'!$B$44/$A22+'9. Valuation'!$B$45/D$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>159.070475767008</v>
+      </c>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="78" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="F23" s="21" t="s">
-        <v>415</v>
-      </c>
+      <c r="A23" s="79" t="n">
+        <v>0.0525</v>
+      </c>
+      <c r="B23" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A23+'9. Valuation'!$B$43/$A23+'9. Valuation'!$B$44/$A23+'9. Valuation'!$B$45/B$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>152.730575782599</v>
+      </c>
+      <c r="C23" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A23+'9. Valuation'!$B$43/$A23+'9. Valuation'!$B$44/$A23+'9. Valuation'!$B$45/C$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>151.095788604459</v>
+      </c>
+      <c r="D23" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A23+'9. Valuation'!$B$43/$A23+'9. Valuation'!$B$44/$A23+'9. Valuation'!$B$45/D$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>149.712507146033</v>
+      </c>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="78" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="F24" s="21" t="s">
-        <v>415</v>
-      </c>
+      <c r="A24" s="79" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="B24" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A24+'9. Valuation'!$B$43/$A24+'9. Valuation'!$B$44/$A24+'9. Valuation'!$B$45/B$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>144.223331581713</v>
+      </c>
+      <c r="C24" s="81" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A24+'9. Valuation'!$B$43/$A24+'9. Valuation'!$B$44/$A24+'9. Valuation'!$B$45/C$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>142.588544403573</v>
+      </c>
+      <c r="D24" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A24+'9. Valuation'!$B$43/$A24+'9. Valuation'!$B$44/$A24+'9. Valuation'!$B$45/D$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>141.205262945147</v>
+      </c>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="78" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="B25" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="F25" s="21" t="s">
-        <v>415</v>
-      </c>
+      <c r="A25" s="79" t="n">
+        <v>0.0575</v>
+      </c>
+      <c r="B25" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A25+'9. Valuation'!$B$43/$A25+'9. Valuation'!$B$44/$A25+'9. Valuation'!$B$45/B$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>136.455847746122</v>
+      </c>
+      <c r="C25" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A25+'9. Valuation'!$B$43/$A25+'9. Valuation'!$B$44/$A25+'9. Valuation'!$B$45/C$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>134.821060567982</v>
+      </c>
+      <c r="D25" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A25+'9. Valuation'!$B$43/$A25+'9. Valuation'!$B$44/$A25+'9. Valuation'!$B$45/D$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>133.437779109556</v>
+      </c>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="78" t="n">
+      <c r="A26" s="79" t="n">
         <v>0.06</v>
       </c>
-      <c r="B26" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="E26" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="F26" s="21" t="s">
-        <v>415</v>
-      </c>
+      <c r="B26" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A26+'9. Valuation'!$B$43/$A26+'9. Valuation'!$B$44/$A26+'9. Valuation'!$B$45/B$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>129.335654230163</v>
+      </c>
+      <c r="C26" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A26+'9. Valuation'!$B$43/$A26+'9. Valuation'!$B$44/$A26+'9. Valuation'!$B$45/C$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>127.700867052023</v>
+      </c>
+      <c r="D26" s="80" t="n">
+        <f aca="false">('9. Valuation'!$B$42/$A26+'9. Valuation'!$B$43/$A26+'9. Valuation'!$B$44/$A26+'9. Valuation'!$B$45/D$21+'9. Valuation'!$D$49+'9. Valuation'!$D$50-'9. Valuation'!$D$51-'9. Valuation'!$D$52)/'9. Valuation'!$D$55</f>
+        <v>126.317585593597</v>
+      </c>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B31" s="20"/>
       <c r="C31" s="20"/>
@@ -3997,56 +4021,56 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>417</v>
-      </c>
-      <c r="B33" s="81" t="n">
+        <v>415</v>
+      </c>
+      <c r="B33" s="82" t="n">
         <f aca="false">'9. Valuation'!B66</f>
-        <v>172.88</v>
+        <v>203.62</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>418</v>
-      </c>
-      <c r="B34" s="81" t="n">
+        <v>416</v>
+      </c>
+      <c r="B34" s="82" t="n">
         <f aca="false">'9. Valuation'!B64</f>
-        <v>104.17664341158</v>
+        <v>119.887201556513</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>419</v>
-      </c>
-      <c r="B35" s="81" t="n">
+        <v>417</v>
+      </c>
+      <c r="B35" s="82" t="n">
         <f aca="false">'9. Valuation'!B65</f>
-        <v>113.220860064791</v>
+        <v>142.588544403573</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>420</v>
-      </c>
-      <c r="B36" s="81" t="n">
+        <v>418</v>
+      </c>
+      <c r="B36" s="82" t="n">
         <f aca="false">'9. Valuation'!B68</f>
-        <v>108.698751738185</v>
+        <v>131.237872980043</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>421</v>
-      </c>
-      <c r="B37" s="68" t="n">
+        <v>419</v>
+      </c>
+      <c r="B37" s="67" t="n">
         <f aca="false">'9. Valuation'!B70</f>
-        <v>-0.37124738698412</v>
+        <v>-0.355476510264005</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
         <v>405</v>
       </c>
-      <c r="B38" s="82" t="str">
+      <c r="B38" s="83" t="str">
         <f aca="false">'9. Valuation'!B72</f>
-        <v>[Buy / Hold / Sell — your call, based on the model output + your thesis]</v>
+        <v>HOLD — ~55% premium to stabilized intrinsic (~$131 blended: DCF ~$120, NAV ~$143) with no margin of safety even at the generous corners. The premium reflects development-pipeline and AI-growth optionality a stabilized model excludes; quality asset and structural demand argue for accumulating on power-driven weakness, not chasing at the highs.</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4054,26 +4078,26 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B40" s="43" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B41" s="43" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B42" s="43" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -4210,7 +4234,7 @@
         <v>136</v>
       </c>
       <c r="B9" s="22" t="n">
-        <v>0.055</v>
+        <v>0.05</v>
       </c>
       <c r="L9" s="15" t="s">
         <v>137</v>
@@ -4221,7 +4245,7 @@
         <v>138</v>
       </c>
       <c r="B10" s="23" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="L10" s="15" t="s">
         <v>139</v>
@@ -4472,7 +4496,7 @@
       </c>
       <c r="L27" s="15"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>158</v>
       </c>
@@ -4517,7 +4541,7 @@
       </c>
       <c r="B31" s="27" t="n">
         <f aca="false">B8+B10*B9</f>
-        <v>0.1055</v>
+        <v>0.095</v>
       </c>
       <c r="L31" s="15" t="s">
         <v>162</v>
@@ -4551,7 +4575,7 @@
       </c>
       <c r="B34" s="27" t="n">
         <f aca="false">(1-B33)*B31+B33*B32</f>
-        <v>0.078275</v>
+        <v>0.0725</v>
       </c>
       <c r="L34" s="15" t="s">
         <v>168</v>
@@ -4562,7 +4586,7 @@
         <v>169</v>
       </c>
       <c r="B35" s="28" t="n">
-        <v>0.065</v>
+        <v>0.0575</v>
       </c>
       <c r="L35" s="15" t="s">
         <v>170</v>
@@ -4573,7 +4597,7 @@
         <v>171</v>
       </c>
       <c r="B36" s="28" t="n">
-        <v>0.065</v>
+        <v>0.055</v>
       </c>
       <c r="L36" s="15" t="s">
         <v>172</v>
@@ -4588,7 +4612,7 @@
       </c>
       <c r="L37" s="15"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
         <v>174</v>
       </c>
@@ -4599,7 +4623,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>176</v>
       </c>
@@ -5556,7 +5580,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="39" t="s">
         <v>257</v>
       </c>
@@ -6215,7 +6239,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="44" t="s">
         <v>280</v>
       </c>
@@ -7842,7 +7866,7 @@
         <v>7.39</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="M6" s="1" t="s">
         <v>322</v>
       </c>
@@ -7871,7 +7895,7 @@
         <v>4.88</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="M8" s="1" t="s">
         <v>325</v>
       </c>
@@ -8632,7 +8656,7 @@
       <c r="C51" s="59"/>
       <c r="D51" s="59"/>
       <c r="E51" s="59"/>
-      <c r="F51" s="64" t="n">
+      <c r="F51" s="51" t="n">
         <v>4.88</v>
       </c>
       <c r="G51" s="59"/>
@@ -8645,89 +8669,89 @@
       <c r="A53" s="57" t="s">
         <v>356</v>
       </c>
-      <c r="B53" s="65" t="n">
+      <c r="B53" s="64" t="n">
         <f aca="false">IFERROR(B51/B49,0)</f>
         <v>0</v>
       </c>
-      <c r="C53" s="65" t="n">
+      <c r="C53" s="64" t="n">
         <f aca="false">IFERROR(C51/C49,0)</f>
         <v>0</v>
       </c>
-      <c r="D53" s="65" t="n">
+      <c r="D53" s="64" t="n">
         <f aca="false">IFERROR(D51/D49,0)</f>
         <v>0</v>
       </c>
-      <c r="E53" s="65" t="n">
+      <c r="E53" s="64" t="n">
         <f aca="false">IFERROR(E51/E49,0)</f>
         <v>0</v>
       </c>
-      <c r="F53" s="65" t="n">
+      <c r="F53" s="64" t="n">
         <f aca="false">IFERROR(F51/F49,0)</f>
         <v>0</v>
       </c>
-      <c r="G53" s="65" t="n">
+      <c r="G53" s="64" t="n">
         <f aca="false">IFERROR(G51/G49,0)</f>
         <v>0</v>
       </c>
-      <c r="H53" s="65" t="n">
+      <c r="H53" s="64" t="n">
         <f aca="false">IFERROR(H51/H49,0)</f>
         <v>0</v>
       </c>
-      <c r="I53" s="65" t="n">
+      <c r="I53" s="64" t="n">
         <f aca="false">IFERROR(I51/I49,0)</f>
         <v>0</v>
       </c>
-      <c r="J53" s="65" t="n">
+      <c r="J53" s="64" t="n">
         <f aca="false">IFERROR(J51/J49,0)</f>
         <v>0</v>
       </c>
-      <c r="K53" s="65" t="n">
+      <c r="K53" s="64" t="n">
         <f aca="false">IFERROR(K51/K49,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="66" t="s">
+      <c r="A56" s="65" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="67" t="s">
+      <c r="A57" s="66" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="67" t="s">
+      <c r="A58" s="66" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="67" t="s">
+      <c r="A59" s="66" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="67" t="s">
+      <c r="A60" s="66" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="67" t="s">
+      <c r="A61" s="66" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="67" t="s">
+      <c r="A62" s="66" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="67" t="s">
+      <c r="A63" s="66" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="67" t="s">
+      <c r="A64" s="66" t="s">
         <v>365</v>
       </c>
     </row>

</xml_diff>